<commit_message>
feat(backend): unified single-sheet Excel layout + per-type explore stats
* Excel ingestion accepts a single Node/Edge/Graph sheet with a Type column;
  per-type DataFrames are split via Parameter-sheet declarations and unrelated
  feature columns are dropped so each slice only carries its own features.
* compute_generic_explore takes per-type node_dfs/edge_dfs and reports
  missing counts against the type's own row count, removing the false
  ~66% missing readings on heterogeneous uploads.
* Demo generator emits the new layout; v2 demo workbooks regenerated.
* Legacy per-type sheets (Node_cell, Edge_pin2pin, ...) still parse for
  backwards compatibility.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/demo_data/demo_multigraph_homo.v2.xlsx
+++ b/backend/demo_data/demo_multigraph_homo.v2.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Node_default" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Edge_default" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Graph_default" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Node" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Edge" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Graph" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Edge_Type</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -68610,7 +68610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68621,10 +68621,15 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>num_cells</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>target_delay</t>
         </is>
@@ -68634,10 +68639,15 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>40</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>35.216</v>
       </c>
     </row>
@@ -68645,10 +68655,15 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>38</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>35.205</v>
       </c>
     </row>
@@ -68656,10 +68671,15 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>38</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>33.152</v>
       </c>
     </row>
@@ -68667,10 +68687,15 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>21</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>28.74</v>
       </c>
     </row>
@@ -68678,10 +68703,15 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>44</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>30.758</v>
       </c>
     </row>
@@ -68689,10 +68719,15 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>26</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>33.87</v>
       </c>
     </row>
@@ -68700,10 +68735,15 @@
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>49</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>28.443</v>
       </c>
     </row>
@@ -68711,10 +68751,15 @@
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>38</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>36.663</v>
       </c>
     </row>
@@ -68722,10 +68767,15 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>40</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>31.184</v>
       </c>
     </row>
@@ -68733,10 +68783,15 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>28</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>33.795</v>
       </c>
     </row>
@@ -68744,10 +68799,15 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>47</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>34.855</v>
       </c>
     </row>
@@ -68755,10 +68815,15 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>40</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>34.261</v>
       </c>
     </row>
@@ -68766,10 +68831,15 @@
       <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>43</v>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>30.712</v>
       </c>
     </row>
@@ -68777,10 +68847,15 @@
       <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
         <v>45</v>
       </c>
-      <c r="C15" t="n">
+      <c r="D15" t="n">
         <v>34.628</v>
       </c>
     </row>
@@ -68788,10 +68863,15 @@
       <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
         <v>26</v>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>27.627</v>
       </c>
     </row>
@@ -68799,10 +68879,15 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>47</v>
       </c>
-      <c r="C17" t="n">
+      <c r="D17" t="n">
         <v>32.819</v>
       </c>
     </row>
@@ -68810,10 +68895,15 @@
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>26</v>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>26.929</v>
       </c>
     </row>
@@ -68821,10 +68911,15 @@
       <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>47</v>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>33.96</v>
       </c>
     </row>
@@ -68832,10 +68927,15 @@
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
         <v>38</v>
       </c>
-      <c r="C20" t="n">
+      <c r="D20" t="n">
         <v>29.898</v>
       </c>
     </row>
@@ -68843,10 +68943,15 @@
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
         <v>42</v>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="n">
         <v>32.733</v>
       </c>
     </row>
@@ -68854,10 +68959,15 @@
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
         <v>48</v>
       </c>
-      <c r="C22" t="n">
+      <c r="D22" t="n">
         <v>36.096</v>
       </c>
     </row>
@@ -68865,10 +68975,15 @@
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
         <v>41</v>
       </c>
-      <c r="C23" t="n">
+      <c r="D23" t="n">
         <v>27.236</v>
       </c>
     </row>
@@ -68876,10 +68991,15 @@
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
         <v>22</v>
       </c>
-      <c r="C24" t="n">
+      <c r="D24" t="n">
         <v>37.506</v>
       </c>
     </row>
@@ -68887,10 +69007,15 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
         <v>50</v>
       </c>
-      <c r="C25" t="n">
+      <c r="D25" t="n">
         <v>38.494</v>
       </c>
     </row>
@@ -68898,10 +69023,15 @@
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
         <v>36</v>
       </c>
-      <c r="C26" t="n">
+      <c r="D26" t="n">
         <v>31.415</v>
       </c>
     </row>
@@ -68909,10 +69039,15 @@
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
         <v>44</v>
       </c>
-      <c r="C27" t="n">
+      <c r="D27" t="n">
         <v>35.929</v>
       </c>
     </row>
@@ -68920,10 +69055,15 @@
       <c r="A28" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
         <v>28</v>
       </c>
-      <c r="C28" t="n">
+      <c r="D28" t="n">
         <v>39.458</v>
       </c>
     </row>
@@ -68931,10 +69071,15 @@
       <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
         <v>38</v>
       </c>
-      <c r="C29" t="n">
+      <c r="D29" t="n">
         <v>26.56</v>
       </c>
     </row>
@@ -68942,10 +69087,15 @@
       <c r="A30" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
         <v>35</v>
       </c>
-      <c r="C30" t="n">
+      <c r="D30" t="n">
         <v>36.564</v>
       </c>
     </row>
@@ -68953,10 +69103,15 @@
       <c r="A31" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
         <v>27</v>
       </c>
-      <c r="C31" t="n">
+      <c r="D31" t="n">
         <v>37.341</v>
       </c>
     </row>

</xml_diff>